<commit_message>
Update the project for all three stacks across five time frames
</commit_message>
<xml_diff>
--- a/logs/experiment_log.xlsx
+++ b/logs/experiment_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z0051rra\Downloads\Neurofind Project\logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2107E2F2-58DD-49F2-90E7-EBAC2B492777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF39A04-527D-4311-9AD1-52E6F349E298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11790" yWindow="10800" windowWidth="19420" windowHeight="10300" xr2:uid="{F9776EC4-E5BF-4E5D-8A0A-73F1CB30A0CB}"/>
+    <workbookView xWindow="28680" yWindow="-1860" windowWidth="29040" windowHeight="17520" xr2:uid="{F9776EC4-E5BF-4E5D-8A0A-73F1CB30A0CB}"/>
   </bookViews>
   <sheets>
     <sheet name="experiments_log" sheetId="1" r:id="rId1"/>
@@ -20,67 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
-  <si>
-    <t>experiment_id</t>
-  </si>
-  <si>
-    <t>Ex1</t>
-  </si>
-  <si>
-    <t>12.06.2026</t>
-  </si>
-  <si>
-    <t>Purpose</t>
-  </si>
-  <si>
-    <t>Input</t>
-  </si>
-  <si>
-    <t>Output</t>
-  </si>
-  <si>
-    <t>Metrics</t>
-  </si>
-  <si>
-    <t>Result</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>number_of_candidates_searched; 
-runtime_seconds;
-distance_to_target;</t>
-  </si>
-  <si>
-    <t>Evaluate full search vs local search using human-labeled stack1 and stack2 frame-0 pairs</t>
-  </si>
-  <si>
-    <t>15  label pairs;
-stack2 test candidate points;
-stack2 test embeddings;
-test size = 1000</t>
-  </si>
-  <si>
-    <t>Ex1_local_search_results_stack1_stack2_test.csv</t>
-  </si>
-  <si>
-    <t>Pipeline runs on label pairs; predictions are far from target in given subset.</t>
-  </si>
-  <si>
-    <t>Uses only first 1000 stack2 candidates and embeddings and not full candidate set, results are for pipeline validation.</t>
-  </si>
-</sst>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -562,14 +502,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -948,79 +882,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7DFB3CA-602B-465D-B2C4-A0AAF5DCABFC}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.54296875" customWidth="1"/>
-    <col min="2" max="2" width="11.81640625" customWidth="1"/>
-    <col min="3" max="3" width="36.453125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="24.08984375" customWidth="1"/>
-    <col min="5" max="5" width="33.6328125" customWidth="1"/>
-    <col min="6" max="6" width="29.90625" customWidth="1"/>
-    <col min="7" max="7" width="24.6328125" customWidth="1"/>
-    <col min="8" max="8" width="17.26953125" customWidth="1"/>
-    <col min="9" max="9" width="26.54296875" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="36.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.140625" customWidth="1"/>
+    <col min="5" max="5" width="33.5703125" customWidth="1"/>
+    <col min="6" max="6" width="29.85546875" customWidth="1"/>
+    <col min="7" max="7" width="24.5703125" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" customWidth="1"/>
+    <col min="9" max="9" width="26.5703125" customWidth="1"/>
   </cols>
-  <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>